<commit_message>
Rename 합의 단가 to 견적단가 on quote screens, printed quote and quote template
Quote item field, detail table, printed quote, past-quote comparison and
the bulk quote template now say 견적단가. Bulk upload still accepts files
using the old '합의판매단가(원)' column header.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/quote.xlsx
+++ b/templates/quote.xlsx
@@ -370,7 +370,7 @@
         <v>수량(개) *</v>
       </c>
       <c r="D1" s="7" t="str">
-        <v>합의판매단가(원) *</v>
+        <v>견적단가(원) *</v>
       </c>
       <c r="E1" s="5" t="str">
         <v>소재ID</v>
@@ -3299,13 +3299,13 @@
     </row>
     <row r="15" ht="64" customHeight="1">
       <c r="A15" s="3" t="str">
-        <v>합의판매단가(원)</v>
+        <v>견적단가(원)</v>
       </c>
       <c r="B15" s="3" t="str">
         <v>필수</v>
       </c>
       <c r="C15" s="3" t="str">
-        <v>합의한 판매단가. 0보다 큰 원 단위 정수입니다.</v>
+        <v>고객에게 제시하는 견적단가. 0보다 큰 원 단위 정수입니다.</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>25000</v>
@@ -3523,7 +3523,7 @@
         <v>선택</v>
       </c>
       <c r="C33" s="3" t="str">
-        <v>원가가산률 / 매출이익률; 추천만 계산하고 합의판매단가는 바꾸지 않음</v>
+        <v>원가가산률 / 매출이익률; 추천만 계산하고 견적단가는 바꾸지 않음</v>
       </c>
       <c r="D33" s="6" t="str"/>
     </row>
@@ -3600,7 +3600,7 @@
         <v>수량(개) *</v>
       </c>
       <c r="D1" s="5" t="str">
-        <v>합의판매단가(원) *</v>
+        <v>견적단가(원) *</v>
       </c>
       <c r="E1" s="5" t="str">
         <v>소재ID</v>

</xml_diff>